<commit_message>
feat: inclusão de métrica Média de Itens por Compra
</commit_message>
<xml_diff>
--- a/data_processed/metricas_consolidadas.xlsx
+++ b/data_processed/metricas_consolidadas.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Total Transações" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Faturamento Por Tipo Consumo" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Análise Temporal" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Média de Itens por Compra" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -993,4 +994,40 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Métrica</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Média de itens por compra</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: inclusão de métrica percentual de nulos por coluna
</commit_message>
<xml_diff>
--- a/data_processed/metricas_consolidadas.xlsx
+++ b/data_processed/metricas_consolidadas.xlsx
@@ -15,6 +15,7 @@
     <sheet name="Faturamento Por Tipo Consumo" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Análise Temporal" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Média de Itens por Compra" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Percentual de nulos por coluna" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1030,4 +1031,126 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Coluna</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Porcentagem Nulos</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Cod_Transacao</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Produto</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>9.68%</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Quantidade</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>4.79%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Preço Unitário</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>5.33%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Valor Total</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Forma de Pagamento</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>31.75%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Tipo de Consumo</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>39.58%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Data da Transação</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>4.60%</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: inclusão de quarentena para dados sem data
</commit_message>
<xml_diff>
--- a/data_processed/metricas_consolidadas.xlsx
+++ b/data_processed/metricas_consolidadas.xlsx
@@ -16,6 +16,7 @@
     <sheet name="Análise Temporal" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Média de Itens por Compra" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Percentual de nulos por coluna" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Contagem de registros duplicado" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -475,11 +476,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3090</v>
+        <v>2946</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>R$ 3.223,00</t>
+          <t>R$ 3.067,00</t>
         </is>
       </c>
     </row>
@@ -490,11 +491,11 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3333</v>
+        <v>3147</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>R$ 10.407,00</t>
+          <t>R$ 9.837,00</t>
         </is>
       </c>
     </row>
@@ -505,11 +506,11 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3368</v>
+        <v>3251</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>R$ 7.062,00</t>
+          <t>R$ 6.804,00</t>
         </is>
       </c>
     </row>
@@ -520,11 +521,11 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3157</v>
+        <v>2978</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>R$ 4.956,00</t>
+          <t>R$ 4.660,50</t>
         </is>
       </c>
     </row>
@@ -580,11 +581,11 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3310</v>
+        <v>3161</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>R$ 17.320,00</t>
+          <t>R$ 16.550,00</t>
         </is>
       </c>
     </row>
@@ -595,11 +596,11 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>3249</v>
+        <v>3093</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>R$ 13.680,00</t>
+          <t>R$ 13.032,00</t>
         </is>
       </c>
     </row>
@@ -610,11 +611,11 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3373</v>
+        <v>3216</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>R$ 10.509,00</t>
+          <t>R$ 10.017,00</t>
         </is>
       </c>
     </row>
@@ -625,12 +626,48 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3221</v>
+        <v>3085</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>R$ 13.320,00</t>
-        </is>
+          <t>R$ 12.760,00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Métrica</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Total de Registros Duplicados</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -667,7 +704,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>R$ 89,016.00</t>
+          <t>R$ 84,850.50</t>
         </is>
       </c>
     </row>
@@ -710,11 +747,11 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>R$ 20.385,50</t>
+          <t>R$ 19.514,50</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>2292</v>
+        <v>2198</v>
       </c>
     </row>
     <row r="3">
@@ -725,11 +762,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>R$ 20.443,50</t>
+          <t>R$ 19.473,00</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2276</v>
+        <v>2173</v>
       </c>
     </row>
     <row r="4">
@@ -740,11 +777,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>R$ 20.412,00</t>
+          <t>R$ 19.540,50</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2263</v>
+        <v>2163</v>
       </c>
     </row>
   </sheetData>
@@ -781,7 +818,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>R$ 8.90</t>
+          <t>R$ 8.89</t>
         </is>
       </c>
     </row>
@@ -818,7 +855,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>10002</v>
+        <v>9542</v>
       </c>
     </row>
   </sheetData>
@@ -860,11 +897,11 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>R$ 26.513,00</t>
+          <t>R$ 25.347,00</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3027</v>
+        <v>2894</v>
       </c>
     </row>
     <row r="3">
@@ -875,11 +912,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>R$ 27.149,50</t>
+          <t>R$ 25.861,00</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>3020</v>
+        <v>2875</v>
       </c>
     </row>
   </sheetData>
@@ -1074,7 +1111,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>9.68%</t>
+          <t>9.71%</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1123,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>4.79%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -1098,7 +1135,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>5.33%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -1122,7 +1159,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>31.75%</t>
+          <t>31.57%</t>
         </is>
       </c>
     </row>
@@ -1134,7 +1171,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>39.58%</t>
+          <t>39.59%</t>
         </is>
       </c>
     </row>
@@ -1146,7 +1183,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>4.60%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: inclusão de novos dados brutos
</commit_message>
<xml_diff>
--- a/data_processed/metricas_consolidadas.xlsx
+++ b/data_processed/metricas_consolidadas.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -577,58 +577,73 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SALADA</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3161</v>
+        <v>2622</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>R$ 16.550,00</t>
+          <t>R$ 8.091,50</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SANDUICHE</t>
+          <t>SALADA</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>3093</v>
+        <v>3161</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>R$ 13.032,00</t>
+          <t>R$ 16.550,00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SUCO</t>
+          <t>SANDUICHE</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3216</v>
+        <v>3093</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>R$ 10.017,00</t>
+          <t>R$ 13.032,00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>SUCO</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>3216</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>R$ 10.017,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>VITAMINA</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="B14" t="n">
         <v>3085</v>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>R$ 12.760,00</t>
         </is>
@@ -719,7 +734,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -782,6 +797,21 @@
       </c>
       <c r="C4" t="n">
         <v>2163</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>R$ 26.322,50</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>3015</v>
       </c>
     </row>
   </sheetData>
@@ -869,7 +899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -892,30 +922,45 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PARA VIAGEM</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>R$ 25.347,00</t>
+          <t>R$ 33.642,50</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>2894</v>
+        <v>3780</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>PARA VIAGEM</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>R$ 25.347,00</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2894</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>PRESENCIAL</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>R$ 25.861,00</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="C4" t="n">
         <v>2875</v>
       </c>
     </row>
@@ -1076,7 +1121,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1111,7 +1156,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>9.71%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -1123,7 +1168,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>4.75%</t>
         </is>
       </c>
     </row>
@@ -1135,7 +1180,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>5.30%</t>
         </is>
       </c>
     </row>
@@ -1147,7 +1192,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0.41%</t>
         </is>
       </c>
     </row>
@@ -1159,7 +1204,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>31.57%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1216,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>39.59%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -1182,6 +1227,42 @@
         </is>
       </c>
       <c r="B9" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>valor_imputado</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>is_valid</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>quality_issues</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>

</xml_diff>

<commit_message>
feat: reformulação dos códigos
</commit_message>
<xml_diff>
--- a/data_processed/metricas_consolidadas.xlsx
+++ b/data_processed/metricas_consolidadas.xlsx
@@ -17,6 +17,7 @@
     <sheet name="Média de Itens por Compra" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Percentual de nulos por coluna" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Contagem de registros duplicado" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Faturamento Agrupado Por ID Pro" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -472,75 +473,75 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BISCOITO</t>
+          <t>CAKE</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2946</v>
+        <v>3143</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>R$ 3.067,00</t>
+          <t>R$ 9.825,00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BOLO</t>
+          <t>COFFEE</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3147</v>
+        <v>3251</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>R$ 9.837,00</t>
+          <t>R$ 6.804,00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CAFÉ</t>
+          <t>COOKIE</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3251</v>
+        <v>2946</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>R$ 6.804,00</t>
+          <t>R$ 3.067,00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CHÁ</t>
+          <t>ESPRESSO</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2978</v>
+        <v>1</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>R$ 4.660,50</t>
+          <t>R$ 2,50</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>EXPRESSO</t>
+          <t>JUICE</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>3216</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>R$ 2,50</t>
+          <t>R$ 10.017,00</t>
         </is>
       </c>
     </row>
@@ -551,11 +552,11 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>R$ 14,00</t>
+          <t>R$ 7,00</t>
         </is>
       </c>
     </row>
@@ -581,18 +582,18 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2622</v>
+        <v>217092</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>R$ 8.091,50</t>
+          <t>R$ 706.903,83</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SALADA</t>
+          <t>SALAD</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -607,45 +608,45 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SANDUICHE</t>
+          <t>SANDWICH</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3093</v>
+        <v>3089</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>R$ 13.032,00</t>
+          <t>R$ 13.016,00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SUCO</t>
+          <t>SMOOTHIE</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3216</v>
+        <v>3085</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>R$ 10.017,00</t>
+          <t>R$ 12.760,00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>VITAMINA</t>
+          <t>TEA</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3085</v>
+        <v>2978</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>R$ 12.760,00</t>
+          <t>R$ 4.660,50</t>
         </is>
       </c>
     </row>
@@ -682,7 +683,1078 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C81"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Cod_Produto</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Quantidade</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Valor Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="n">
+        <v>214</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>R$ 3.852,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="n">
+        <v>183</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>R$ 3.294,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="n">
+        <v>169</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>R$ 2.492,75</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="n">
+        <v>150</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>R$ 3.067,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="n">
+        <v>148</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>R$ 2.220,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="n">
+        <v>218</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>R$ 4.578,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
         <v>7</v>
+      </c>
+      <c r="B8" t="n">
+        <v>146</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>R$ 2.883,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="n">
+        <v>260</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>R$ 11.700,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="n">
+        <v>206</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>R$ 4.657,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="n">
+        <v>134</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>R$ 1.340,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="n">
+        <v>152</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>R$ 1.360,40</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="n">
+        <v>153</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>R$ 1.369,35</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="n">
+        <v>161</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>R$ 1.440,95</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="n">
+        <v>142</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>R$ 1.270,90</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="n">
+        <v>159</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>R$ 1.470,75</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="n">
+        <v>153</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>R$ 1.369,35</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="n">
+        <v>168</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>R$ 1.596,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="n">
+        <v>122</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>R$ 1.335,90</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="n">
+        <v>118</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>R$ 755,20</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="n">
+        <v>221</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>R$ 1.679,60</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="n">
+        <v>148</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>R$ 1.972,84</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="n">
+        <v>4484</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>R$ 8.968,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="n">
+        <v>4410</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>R$ 11.025,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="n">
+        <v>3997</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>R$ 11.991,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="n">
+        <v>4310</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>R$ 9.482,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="n">
+        <v>4385</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>R$ 13.155,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="n">
+        <v>4317</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>R$ 15.109,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="n">
+        <v>4178</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>R$ 8.356,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="n">
+        <v>4547</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>R$ 11.367,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="n">
+        <v>4195</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>R$ 12.585,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="n">
+        <v>4433</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>R$ 9.752,60</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="n">
+        <v>4393</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>R$ 13.179,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="n">
+        <v>4227</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>R$ 14.794,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="n">
+        <v>4018</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>R$ 9.844,10</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="n">
+        <v>4018</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>R$ 12.455,80</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="n">
+        <v>4395</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>R$ 16.481,25</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="n">
+        <v>4165</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>R$ 12.495,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="n">
+        <v>4602</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>R$ 17.257,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="n">
+        <v>4497</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>R$ 19.112,25</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="n">
+        <v>4266</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>R$ 15.997,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="n">
+        <v>4151</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>R$ 17.641,75</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="n">
+        <v>4325</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>R$ 10.812,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="n">
+        <v>4089</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>R$ 12.267,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="n">
+        <v>4564</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>R$ 11.410,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="n">
+        <v>4350</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>R$ 13.050,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="n">
+        <v>4477</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>R$ 11.192,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="n">
+        <v>4220</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>R$ 12.660,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="n">
+        <v>4200</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>R$ 10.500,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="n">
+        <v>4309</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>R$ 12.927,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="n">
+        <v>4708</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>R$ 11.770,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="n">
+        <v>4245</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>R$ 12.735,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="n">
+        <v>4512</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>R$ 11.280,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="n">
+        <v>4174</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>R$ 12.522,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="n">
+        <v>4643</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>R$ 11.607,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="n">
+        <v>4346</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>R$ 17.384,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" t="n">
+        <v>4171</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>R$ 10.636,05</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" t="n">
+        <v>4404</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>R$ 13.652,40</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" t="n">
+        <v>4007</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>R$ 14.024,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" t="n">
+        <v>4668</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>R$ 21.006,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" t="n">
+        <v>4329</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>R$ 16.233,75</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" t="n">
+        <v>4453</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>R$ 21.151,75</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>63</v>
+      </c>
+      <c r="B63" t="n">
+        <v>2576</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>R$ 2.060,80</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>64</v>
+      </c>
+      <c r="B64" t="n">
+        <v>2372</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>R$ 1.897,60</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>65</v>
+      </c>
+      <c r="B65" t="n">
+        <v>2905</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>R$ 2.324,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>69</v>
+      </c>
+      <c r="B66" t="n">
+        <v>2028</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>R$ 6.608,01</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>70</v>
+      </c>
+      <c r="B67" t="n">
+        <v>2092</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>R$ 6.818,44</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>71</v>
+      </c>
+      <c r="B68" t="n">
+        <v>3096</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>R$ 11.625,98</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>72</v>
+      </c>
+      <c r="B69" t="n">
+        <v>2540</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>R$ 8.011,61</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>73</v>
+      </c>
+      <c r="B70" t="n">
+        <v>1911</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>R$ 7.168,13</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>74</v>
+      </c>
+      <c r="B71" t="n">
+        <v>1836</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>R$ 6.436,56</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>75</v>
+      </c>
+      <c r="B72" t="n">
+        <v>1954</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>R$ 6.861,88</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>76</v>
+      </c>
+      <c r="B73" t="n">
+        <v>1924</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>R$ 6.748,96</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>77</v>
+      </c>
+      <c r="B74" t="n">
+        <v>1820</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>R$ 5.460,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>78</v>
+      </c>
+      <c r="B75" t="n">
+        <v>1985</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>R$ 8.949,45</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>79</v>
+      </c>
+      <c r="B76" t="n">
+        <v>2028</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>R$ 7.626,62</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>81</v>
+      </c>
+      <c r="B77" t="n">
+        <v>221</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>R$ 6.163,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>82</v>
+      </c>
+      <c r="B78" t="n">
+        <v>240</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>R$ 2.935,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>83</v>
+      </c>
+      <c r="B79" t="n">
+        <v>315</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>R$ 4.509,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>84</v>
+      </c>
+      <c r="B80" t="n">
+        <v>2658</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>R$ 2.126,40</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>87</v>
+      </c>
+      <c r="B81" t="n">
+        <v>3262</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>R$ 8.902,20</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -719,7 +1791,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>R$ 84,850.50</t>
+          <t>R$ 783,627.83</t>
         </is>
       </c>
     </row>
@@ -757,46 +1829,46 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CARTEIRA DIGITAL</t>
+          <t>CASH</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>R$ 19.514,50</t>
+          <t>R$ 19.512,50</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>2198</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CARTÃO DE CRÉDITO</t>
+          <t>CREDIT CARD</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>R$ 19.473,00</t>
+          <t>R$ 19.466,00</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2173</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DINHEIRO</t>
+          <t>DIGITAL WALLET</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>R$ 19.540,50</t>
+          <t>R$ 19.514,50</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2163</v>
+        <v>2198</v>
       </c>
     </row>
     <row r="5">
@@ -807,11 +1879,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>R$ 26.322,50</t>
+          <t>R$ 725.134,83</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>3015</v>
+        <v>152131</v>
       </c>
     </row>
   </sheetData>
@@ -848,7 +1920,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>R$ 8.89</t>
+          <t>R$ 4.94</t>
         </is>
       </c>
     </row>
@@ -885,7 +1957,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>9542</v>
+        <v>158658</v>
       </c>
     </row>
   </sheetData>
@@ -922,46 +1994,46 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>IN-STORE</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>R$ 33.642,50</t>
+          <t>R$ 25.849,00</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3780</v>
+        <v>2874</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PARA VIAGEM</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>R$ 25.347,00</t>
+          <t>R$ 732.438,83</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2894</v>
+        <v>152895</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PRESENCIAL</t>
+          <t>TAKEAWAY</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>R$ 25.861,00</t>
+          <t>R$ 25.340,00</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2875</v>
+        <v>2893</v>
       </c>
     </row>
   </sheetData>
@@ -998,7 +2070,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>R$ 12.139,50</t>
+          <t>R$ 113.816,78</t>
         </is>
       </c>
     </row>
@@ -1010,7 +2082,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>R$ 12.048,50</t>
+          <t>R$ 111.492,44</t>
         </is>
       </c>
     </row>
@@ -1022,7 +2094,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>R$ 11.630,50</t>
+          <t>R$ 111.937,04</t>
         </is>
       </c>
     </row>
@@ -1034,7 +2106,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>R$ 12.394,00</t>
+          <t>R$ 113.161,78</t>
         </is>
       </c>
     </row>
@@ -1046,7 +2118,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>R$ 12.324,50</t>
+          <t>R$ 113.697,50</t>
         </is>
       </c>
     </row>
@@ -1058,7 +2130,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>R$ 12.023,50</t>
+          <t>R$ 108.901,98</t>
         </is>
       </c>
     </row>
@@ -1070,7 +2142,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>R$ 12.290,00</t>
+          <t>R$ 110.620,31</t>
         </is>
       </c>
     </row>
@@ -1107,7 +2179,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1121,7 +2193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1168,7 +2240,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>4.75%</t>
+          <t>0.29%</t>
         </is>
       </c>
     </row>
@@ -1180,7 +2252,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>5.30%</t>
+          <t>0.32%</t>
         </is>
       </c>
     </row>
@@ -1192,7 +2264,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0.41%</t>
+          <t>0.02%</t>
         </is>
       </c>
     </row>
@@ -1235,7 +2307,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>valor_imputado</t>
+          <t>Origem</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1247,22 +2319,118 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>is_valid</t>
+          <t>Hora da Transação</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>6.02%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>Cod_Loja</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>6.02%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Localizacao_Loja</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>6.02%</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Cod_Produto</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>6.02%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Categoria do Produto</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>6.02%</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Tipo do Produto</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>6.02%</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Detalhe do Produto</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>6.02%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>valor_imputado</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>is_valid</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>quality_issues</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>

</xml_diff>